<commit_message>
Update Freiburger Excel: Cornflakes→NOVA 4, remove Bratfett
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/freiburger_nova.xlsx
+++ b/data/freiburger_nova.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\nas-fa0efsusr1\Burgarle\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\Hector-Forschung\Arbeitsordner - Mitarbeiter\Arbeitsordner-Burgard Leonie\3. Paper\BLS\BLS App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{29A5DD45-29BA-4D2B-9D07-A3F39E96F848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A197CD-3F85-433A-98B5-852B54AFCC30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25320" yWindow="4485" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Freiburger Protokoll" sheetId="2" r:id="rId1"/>
@@ -32,12 +32,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="207">
   <si>
     <t>Freiburger Ernährungsprotokoll</t>
   </si>
@@ -655,6 +658,9 @@
   </si>
   <si>
     <t>nicht 4</t>
+  </si>
+  <si>
+    <t>PRINZIP:Foods were classified according to their most common form of consumption in the general population, with preference for minimally processed or home-prepared equivalents where applicable.</t>
   </si>
 </sst>
 </file>
@@ -684,12 +690,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -704,7 +716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -716,6 +728,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -996,22 +1012,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D29C704-C0F2-47D5-B55F-40B84D8C929C}">
-  <dimension ref="A1:F194"/>
+  <dimension ref="A1:G194"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.85546875" style="3" customWidth="1"/>
     <col min="2" max="2" width="11.42578125" style="3"/>
     <col min="3" max="3" width="19.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.7109375" style="3" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="3"/>
+    <col min="5" max="6" width="11.42578125" style="3"/>
+    <col min="7" max="7" width="186.5703125" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1026,8 +1044,11 @@
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>72</v>
       </c>
@@ -1037,7 +1058,7 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1053,7 +1074,7 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1069,7 +1090,7 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>74</v>
       </c>
@@ -1085,7 +1106,7 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>75</v>
       </c>
@@ -1101,7 +1122,7 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1117,7 +1138,7 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>76</v>
       </c>
@@ -1133,7 +1154,7 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1149,7 +1170,7 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1165,7 +1186,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>77</v>
       </c>
@@ -1181,7 +1202,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1197,7 +1218,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>71</v>
       </c>
@@ -1207,7 +1228,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
@@ -1223,7 +1244,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1659,8 +1680,8 @@
       <c r="C43" s="1">
         <v>4</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>205</v>
+      <c r="D43" s="7">
+        <v>4</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -3036,7 +3057,7 @@
         <v>10</v>
       </c>
       <c r="D132" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>

</xml_diff>